<commit_message>
feat: add to_machine column to shikake shield
Add a To Machine field to the shikake shield master data, mirroring the
bonder/joint processes (placed right after blade).

- migration: add nullable to_machine after blade on master_shikake_shield
- model: add to_machine to fillable
- template config: add 'To Machine' header to getShieldHeaders
- import: map to_machine; bump shield assy start column 24 -> 25
- request: validate process_data.to_machine
- edit/detail modal + index JS: input, display row and populate logic
- regenerate shikake Excel templates so the downloadable Shield template
  includes the new column (import validates headers strictly)
</commit_message>
<xml_diff>
--- a/public/docs/Template_Shikake_Shield.xlsx
+++ b/public/docs/Template_Shikake_Shield.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
   <si>
     <t>Carline</t>
   </si>
@@ -45,6 +45,9 @@
   </si>
   <si>
     <t>Blade</t>
+  </si>
+  <si>
+    <t>To Machine</t>
   </si>
   <si>
     <t>QRCode Drawing</t>
@@ -459,7 +462,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="11.569" bestFit="true" customWidth="true" style="0"/>
@@ -472,12 +475,12 @@
     <col min="8" max="8" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="9" max="9" width="11.569" bestFit="true" customWidth="true" style="0"/>
     <col min="10" max="10" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="11" max="11" width="19.852" bestFit="true" customWidth="true" style="0"/>
-    <col min="12" max="12" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="13" max="13" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="14" max="14" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="15" max="15" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="16" max="16" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="11" max="11" width="15.139" bestFit="true" customWidth="true" style="0"/>
+    <col min="12" max="12" width="19.852" bestFit="true" customWidth="true" style="0"/>
+    <col min="13" max="13" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="14" max="14" width="13.997" bestFit="true" customWidth="true" style="0"/>
+    <col min="15" max="15" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="16" max="16" width="13.997" bestFit="true" customWidth="true" style="0"/>
     <col min="17" max="17" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="18" max="18" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="19" max="19" width="8.141" bestFit="true" customWidth="true" style="0"/>
@@ -486,9 +489,10 @@
     <col min="22" max="22" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="23" max="23" width="8.141" bestFit="true" customWidth="true" style="0"/>
     <col min="24" max="24" width="8.141" bestFit="true" customWidth="true" style="0"/>
+    <col min="25" max="25" width="8.141" bestFit="true" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
+    <row r="1" spans="1:25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -560,6 +564,9 @@
       </c>
       <c r="X1" s="1" t="s">
         <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>